<commit_message>
Update email app bridge deployment
</commit_message>
<xml_diff>
--- a/email_app/templates/student_lookup_template.xlsx
+++ b/email_app/templates/student_lookup_template.xlsx
@@ -443,15 +443,15 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
@@ -530,12 +530,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>hfnt93@university.ac.uk</t>
+          <t>hfnt93@durham.ac.uk</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hfnt93@university.ac.uk</t>
+          <t>hfnt93@durham.ac.uk</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -550,52 +550,52 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Helen Frost</t>
+          <t>David Chivers</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>123456789</t>
+          <t>Pending Banner</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>BSc Economics</t>
+          <t>Pending Banner</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Undergraduate</t>
+          <t>Pending Banner</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Year 2</t>
+          <t>Pending Banner</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Dr Patel</t>
+          <t>Pending Banner</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://banner.example.edu/student/123456789</t>
+          <t>Pending Banner</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>BNR-123456789</t>
+          <t>Pending Banner</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Provisional test row</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>

</xml_diff>